<commit_message>
Test: Add Auth, Machine API Integration Test
</commit_message>
<xml_diff>
--- a/SOP Deploy.xlsx
+++ b/SOP Deploy.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Data\Drive D\app\Basic App\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2610FDCF-9BBF-4BD4-AC0C-BA43A4A40524}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F674A07-DD7E-496B-9A0D-517EE9728A0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B5F38ADC-63D7-4DD4-8E01-F6FF01CEE954}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="6" xr2:uid="{B5F38ADC-63D7-4DD4-8E01-F6FF01CEE954}"/>
   </bookViews>
   <sheets>
     <sheet name="Overview" sheetId="1" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <sheet name="Docker Prod" sheetId="2" r:id="rId4"/>
     <sheet name="CI CD Main" sheetId="3" r:id="rId5"/>
     <sheet name="SSH Key" sheetId="4" r:id="rId6"/>
-    <sheet name="Gtihub Secret" sheetId="5" r:id="rId7"/>
+    <sheet name="Github Secret" sheetId="5" r:id="rId7"/>
     <sheet name="Droplet" sheetId="6" r:id="rId8"/>
     <sheet name="Deploy SSH" sheetId="7" r:id="rId9"/>
     <sheet name="GHCR Token" sheetId="8" r:id="rId10"/>
@@ -2835,7 +2835,7 @@
     <hyperlink ref="C3" location="'Docker Prod'!A1" display="'Docker Prod'!A1" xr:uid="{BC51C2E0-84BD-40C1-A6D5-333B209C5FA4}"/>
     <hyperlink ref="C4" location="'CI CD Main'!A1" display="สร้าง ci-cd-test.yml" xr:uid="{FFD418BC-61E7-4C3C-9B68-E75E097BFAB3}"/>
     <hyperlink ref="C5" location="'SSH Key'!A1" display="การออก SSH Key" xr:uid="{1EB9A4EE-5B0A-4346-9A9A-C8285ECB3DDB}"/>
-    <hyperlink ref="C6" location="'Gtihub Secret'!A1" display="สร้าง GitHub Secrets" xr:uid="{DB29AED2-38B8-462F-93D3-0503395B6ABE}"/>
+    <hyperlink ref="C6" location="'Github Secret'!A1" display="สร้าง GitHub Secrets" xr:uid="{DB29AED2-38B8-462F-93D3-0503395B6ABE}"/>
     <hyperlink ref="C7" location="Droplet!A1" display="สร้าง Droplet (Digital Ocean)" xr:uid="{7805FCB2-DA0B-4CA8-AEE0-9A199019B40F}"/>
     <hyperlink ref="C8" location="'Deploy SSH'!A1" display="การ Deploy ผ่าน SSH (ครั้งแรก)" xr:uid="{A8B81ADC-84FC-4F15-A118-8E21B78E362B}"/>
     <hyperlink ref="C9" location="'GHCR Token'!A1" display="การออก GHCR Token" xr:uid="{4D734261-3691-48D1-97DF-D14291DBD243}"/>

</xml_diff>